<commit_message>
Update defect 1 and test case links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01WvaaHLHQtm29VcTEU5G3Gz
</commit_message>
<xml_diff>
--- a/Test_Scenarios-Magnus.xlsx
+++ b/Test_Scenarios-Magnus.xlsx
@@ -1345,14 +1345,14 @@
       </c>
       <c r="E5" s="45" t="inlineStr">
         <is>
-          <t>Verify logout</t>
+          <t>Verify logout and the Home page</t>
         </is>
       </c>
       <c r="F5" s="45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">

</xml_diff>